<commit_message>
Fix H2 silkscreen label: 5V -> 3V3
H2 pin 3 is wired to the 3V3 net in v2 but the silkscreen still read 5V.
Re-exported Gerber/BOM/PnP; only the top silkscreen layer changed
(BOM differs only in live LCSC/JLCPCB stock counts).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/fabrication/2026-10-03_v2/BOM_PCB1_1_v2_2026-10-03.xlsx
+++ b/hardware/fabrication/2026-10-03_v2/BOM_PCB1_1_v2_2026-10-03.xlsx
@@ -97,7 +97,7 @@
     <t>2</t>
   </si>
   <si>
-    <t>19195981</t>
+    <t>19193728</t>
   </si>
   <si>
     <t>C15850</t>
@@ -118,7 +118,7 @@
     <t>3</t>
   </si>
   <si>
-    <t>4944805</t>
+    <t>4944583</t>
   </si>
   <si>
     <t>C336792</t>
@@ -163,7 +163,7 @@
     <t>5</t>
   </si>
   <si>
-    <t>979589</t>
+    <t>979535</t>
   </si>
   <si>
     <t>C2937625</t>
@@ -181,7 +181,7 @@
     <t>6</t>
   </si>
   <si>
-    <t>1021657</t>
+    <t>1021650</t>
   </si>
   <si>
     <t>C55528</t>
@@ -223,7 +223,7 @@
     <t>8</t>
   </si>
   <si>
-    <t>3125395</t>
+    <t>3125050</t>
   </si>
   <si>
     <t>C2286</t>
@@ -241,7 +241,7 @@
     <t>9</t>
   </si>
   <si>
-    <t>4812604</t>
+    <t>4812422</t>
   </si>
   <si>
     <t>C5125736</t>
@@ -283,7 +283,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>1374033</t>
+    <t>1374058</t>
   </si>
   <si>
     <t>C25804</t>
@@ -307,7 +307,7 @@
     <t>12</t>
   </si>
   <si>
-    <t>23008358</t>
+    <t>23008785</t>
   </si>
   <si>
     <t>C125627</t>
@@ -349,7 +349,7 @@
     <t>14</t>
   </si>
   <si>
-    <t>7140499</t>
+    <t>7140517</t>
   </si>
   <si>
     <t>C25900</t>
@@ -367,7 +367,7 @@
     <t>15</t>
   </si>
   <si>
-    <t>15448190</t>
+    <t>15448200</t>
   </si>
   <si>
     <t>C2907232</t>
@@ -406,7 +406,7 @@
     <t>17</t>
   </si>
   <si>
-    <t>3408932</t>
+    <t>3408892</t>
   </si>
   <si>
     <t>C25117</t>
@@ -445,7 +445,7 @@
     <t>19</t>
   </si>
   <si>
-    <t>535345</t>
+    <t>535285</t>
   </si>
   <si>
     <t>C2876014</t>
@@ -487,7 +487,7 @@
     <t>21</t>
   </si>
   <si>
-    <t>35033</t>
+    <t>34998</t>
   </si>
   <si>
     <t>C36936554</t>

</xml_diff>